<commit_message>
Fix numeric column formatting in data cleaning example
</commit_message>
<xml_diff>
--- a/examples/04_spreadsheets/data_cleaning/tidy_data.xlsx
+++ b/examples/04_spreadsheets/data_cleaning/tidy_data.xlsx
@@ -471,10 +471,10 @@
           <t>Jan</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n">
-        <v>2001</v>
-      </c>
-      <c r="C2" s="2" t="n">
+      <c r="B2" t="n">
+        <v>2001</v>
+      </c>
+      <c r="C2" t="n">
         <v>2019</v>
       </c>
       <c r="D2" s="2" t="n">
@@ -490,10 +490,10 @@
           <t>Feb</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n">
-        <v>2001</v>
-      </c>
-      <c r="C3" s="2" t="n">
+      <c r="B3" t="n">
+        <v>2001</v>
+      </c>
+      <c r="C3" t="n">
         <v>2019</v>
       </c>
       <c r="D3" s="2" t="n">
@@ -509,10 +509,10 @@
           <t>Mar</t>
         </is>
       </c>
-      <c r="B4" s="2" t="n">
-        <v>2001</v>
-      </c>
-      <c r="C4" s="2" t="n">
+      <c r="B4" t="n">
+        <v>2001</v>
+      </c>
+      <c r="C4" t="n">
         <v>2019</v>
       </c>
       <c r="D4" s="2" t="n">
@@ -528,10 +528,10 @@
           <t>Apr</t>
         </is>
       </c>
-      <c r="B5" s="2" t="n">
-        <v>2001</v>
-      </c>
-      <c r="C5" s="2" t="n">
+      <c r="B5" t="n">
+        <v>2001</v>
+      </c>
+      <c r="C5" t="n">
         <v>2019</v>
       </c>
       <c r="D5" s="2" t="n">
@@ -547,10 +547,10 @@
           <t>May</t>
         </is>
       </c>
-      <c r="B6" s="2" t="n">
-        <v>2001</v>
-      </c>
-      <c r="C6" s="2" t="n">
+      <c r="B6" t="n">
+        <v>2001</v>
+      </c>
+      <c r="C6" t="n">
         <v>2019</v>
       </c>
       <c r="D6" s="2" t="n">
@@ -566,10 +566,10 @@
           <t>Jun</t>
         </is>
       </c>
-      <c r="B7" s="2" t="n">
-        <v>2001</v>
-      </c>
-      <c r="C7" s="2" t="n">
+      <c r="B7" t="n">
+        <v>2001</v>
+      </c>
+      <c r="C7" t="n">
         <v>2019</v>
       </c>
       <c r="D7" s="2" t="n">
@@ -585,10 +585,10 @@
           <t>Jul</t>
         </is>
       </c>
-      <c r="B8" s="2" t="n">
-        <v>2001</v>
-      </c>
-      <c r="C8" s="2" t="n">
+      <c r="B8" t="n">
+        <v>2001</v>
+      </c>
+      <c r="C8" t="n">
         <v>2019</v>
       </c>
       <c r="D8" s="2" t="n">
@@ -604,10 +604,10 @@
           <t>Aug</t>
         </is>
       </c>
-      <c r="B9" s="2" t="n">
-        <v>2001</v>
-      </c>
-      <c r="C9" s="2" t="n">
+      <c r="B9" t="n">
+        <v>2001</v>
+      </c>
+      <c r="C9" t="n">
         <v>2019</v>
       </c>
       <c r="D9" s="2" t="n">
@@ -623,10 +623,10 @@
           <t>Sep</t>
         </is>
       </c>
-      <c r="B10" s="2" t="n">
-        <v>2001</v>
-      </c>
-      <c r="C10" s="2" t="n">
+      <c r="B10" t="n">
+        <v>2001</v>
+      </c>
+      <c r="C10" t="n">
         <v>2019</v>
       </c>
       <c r="D10" s="2" t="n">
@@ -642,10 +642,10 @@
           <t>Oct</t>
         </is>
       </c>
-      <c r="B11" s="2" t="n">
-        <v>2001</v>
-      </c>
-      <c r="C11" s="2" t="n">
+      <c r="B11" t="n">
+        <v>2001</v>
+      </c>
+      <c r="C11" t="n">
         <v>2019</v>
       </c>
       <c r="D11" s="2" t="n">
@@ -661,10 +661,10 @@
           <t>Nov</t>
         </is>
       </c>
-      <c r="B12" s="2" t="n">
-        <v>2001</v>
-      </c>
-      <c r="C12" s="2" t="n">
+      <c r="B12" t="n">
+        <v>2001</v>
+      </c>
+      <c r="C12" t="n">
         <v>2019</v>
       </c>
       <c r="D12" s="2" t="n">
@@ -680,10 +680,10 @@
           <t>Dec</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
-        <v>2001</v>
-      </c>
-      <c r="C13" s="2" t="n">
+      <c r="B13" t="n">
+        <v>2001</v>
+      </c>
+      <c r="C13" t="n">
         <v>2019</v>
       </c>
       <c r="D13" s="2" t="n">

</xml_diff>